<commit_message>
walk through the pooled trait associations and retire the shared analysis functions
</commit_message>
<xml_diff>
--- a/04_Continuous_no_group/01_Trait_Associations/03_Modules/c_data/module_trait_associations.xlsx
+++ b/04_Continuous_no_group/01_Trait_Associations/03_Modules/c_data/module_trait_associations.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5673" uniqueCount="380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5694" uniqueCount="393">
   <si>
     <t>sheet</t>
   </si>
@@ -526,7 +526,7 @@
     <t>phenotype</t>
   </si>
   <si>
-    <t>00_Input/phenotype.csv</t>
+    <t>00_Setup/Input/phenotype.csv</t>
   </si>
   <si>
     <t>5a1989db406daa0b70189a9f0df52cf3</t>
@@ -686,6 +686,15 @@
   </si>
   <si>
     <t>1.7-17</t>
+  </si>
+  <si>
+    <t>enrichVolcano</t>
+  </si>
+  <si>
+    <t>0.3.0.9000</t>
+  </si>
+  <si>
+    <t>Github (Dustyn-T-Lewis/enrichVolcano@d3fed631f4ae95e01bd61137699313f8de5cc86e)</t>
   </si>
   <si>
     <t>evaluate</t>
@@ -868,6 +877,12 @@
     <t>1.0.14</t>
   </si>
   <si>
+    <t>jsonlite</t>
+  </si>
+  <si>
+    <t>2.0.0</t>
+  </si>
+  <si>
     <t>knitr</t>
   </si>
   <si>
@@ -964,6 +979,12 @@
     <t>2.0.3</t>
   </si>
   <si>
+    <t>plyr</t>
+  </si>
+  <si>
+    <t>1.8.9</t>
+  </si>
+  <si>
     <t>png</t>
   </si>
   <si>
@@ -986,6 +1007,9 @@
   </si>
   <si>
     <t>1.2.2</t>
+  </si>
+  <si>
+    <t>2.44.0</t>
   </si>
   <si>
     <t>R6</t>
@@ -1022,6 +1046,9 @@
   </si>
   <si>
     <t>1.2.3</t>
+  </si>
+  <si>
+    <t>reshape2</t>
   </si>
   <si>
     <t>rjson</t>
@@ -1159,10 +1186,22 @@
     <t>3.0.2</t>
   </si>
   <si>
+    <t>writexl</t>
+  </si>
+  <si>
+    <t>2.0.1</t>
+  </si>
+  <si>
     <t>xfun</t>
   </si>
   <si>
     <t>0.57</t>
+  </si>
+  <si>
+    <t>yaml</t>
+  </si>
+  <si>
+    <t>2.3.12</t>
   </si>
 </sst>
 </file>
@@ -1595,7 +1634,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C108"/>
+  <dimension ref="A1:C115"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -1892,15 +1931,15 @@
         <v>222</v>
       </c>
       <c r="C27" t="s">
-        <v>171</v>
+        <v>223</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B28" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C28" t="s">
         <v>171</v>
@@ -1908,13 +1947,13 @@
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B29" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C29" t="s">
-        <v>227</v>
+        <v>171</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -1925,15 +1964,15 @@
         <v>229</v>
       </c>
       <c r="C30" t="s">
-        <v>171</v>
+        <v>230</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B31" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C31" t="s">
         <v>171</v>
@@ -1941,10 +1980,10 @@
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B32" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C32" t="s">
         <v>171</v>
@@ -1952,10 +1991,10 @@
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B33" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C33" t="s">
         <v>171</v>
@@ -1963,10 +2002,10 @@
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B34" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C34" t="s">
         <v>171</v>
@@ -1974,10 +2013,10 @@
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B35" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C35" t="s">
         <v>171</v>
@@ -1985,10 +2024,10 @@
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B36" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C36" t="s">
         <v>171</v>
@@ -1996,10 +2035,10 @@
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B37" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C37" t="s">
         <v>171</v>
@@ -2007,10 +2046,10 @@
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B38" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C38" t="s">
         <v>171</v>
@@ -2018,10 +2057,10 @@
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B39" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C39" t="s">
         <v>171</v>
@@ -2029,10 +2068,10 @@
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C40" t="s">
         <v>171</v>
@@ -2040,10 +2079,10 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B41" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C41" t="s">
         <v>171</v>
@@ -2051,10 +2090,10 @@
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B42" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
       <c r="C42" t="s">
         <v>171</v>
@@ -2062,10 +2101,10 @@
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B43" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="C43" t="s">
         <v>171</v>
@@ -2073,10 +2112,10 @@
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B44" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C44" t="s">
         <v>171</v>
@@ -2084,10 +2123,10 @@
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B45" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C45" t="s">
         <v>171</v>
@@ -2095,10 +2134,10 @@
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B46" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C46" t="s">
         <v>171</v>
@@ -2106,10 +2145,10 @@
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B47" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C47" t="s">
         <v>171</v>
@@ -2117,10 +2156,10 @@
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B48" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C48" t="s">
         <v>171</v>
@@ -2128,10 +2167,10 @@
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B49" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C49" t="s">
         <v>171</v>
@@ -2139,10 +2178,10 @@
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B50" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C50" t="s">
         <v>171</v>
@@ -2150,10 +2189,10 @@
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B51" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C51" t="s">
         <v>171</v>
@@ -2161,10 +2200,10 @@
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B52" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C52" t="s">
         <v>171</v>
@@ -2172,10 +2211,10 @@
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B53" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C53" t="s">
         <v>171</v>
@@ -2183,21 +2222,21 @@
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B54" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C54" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B55" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C55" t="s">
         <v>176</v>
@@ -2205,21 +2244,21 @@
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B56" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C56" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B57" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C57" t="s">
         <v>171</v>
@@ -2227,10 +2266,10 @@
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B58" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C58" t="s">
         <v>171</v>
@@ -2238,10 +2277,10 @@
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B59" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C59" t="s">
         <v>171</v>
@@ -2249,10 +2288,10 @@
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B60" t="s">
-        <v>222</v>
+        <v>289</v>
       </c>
       <c r="C60" t="s">
         <v>171</v>
@@ -2260,21 +2299,21 @@
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B61" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="C61" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B62" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C62" t="s">
         <v>171</v>
@@ -2282,21 +2321,21 @@
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B63" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C63" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B64" t="s">
-        <v>294</v>
+        <v>227</v>
       </c>
       <c r="C64" t="s">
         <v>171</v>
@@ -2304,10 +2343,10 @@
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B65" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C65" t="s">
         <v>171</v>
@@ -2315,10 +2354,10 @@
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B66" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C66" t="s">
         <v>171</v>
@@ -2326,10 +2365,10 @@
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B67" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C67" t="s">
         <v>171</v>
@@ -2337,10 +2376,10 @@
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B68" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C68" t="s">
         <v>171</v>
@@ -2348,10 +2387,10 @@
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B69" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C69" t="s">
         <v>171</v>
@@ -2359,10 +2398,10 @@
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B70" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C70" t="s">
         <v>171</v>
@@ -2370,10 +2409,10 @@
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B71" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C71" t="s">
         <v>171</v>
@@ -2381,10 +2420,10 @@
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B72" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C72" t="s">
         <v>171</v>
@@ -2392,10 +2431,10 @@
     </row>
     <row r="73" spans="1:3">
       <c r="A73" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B73" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C73" t="s">
         <v>171</v>
@@ -2403,10 +2442,10 @@
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B74" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C74" t="s">
         <v>171</v>
@@ -2414,21 +2453,21 @@
     </row>
     <row r="75" spans="1:3">
       <c r="A75" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B75" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C75" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B76" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C76" t="s">
         <v>171</v>
@@ -2436,10 +2475,10 @@
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B77" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C77" t="s">
         <v>171</v>
@@ -2447,21 +2486,21 @@
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B78" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C78" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B79" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C79" t="s">
         <v>171</v>
@@ -2469,10 +2508,10 @@
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B80" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C80" t="s">
         <v>171</v>
@@ -2480,13 +2519,13 @@
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
-        <v>327</v>
+        <v>54</v>
       </c>
       <c r="B81" t="s">
         <v>328</v>
       </c>
       <c r="C81" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
     </row>
     <row r="82" spans="1:3">
@@ -2527,18 +2566,18 @@
         <v>335</v>
       </c>
       <c r="B85" t="s">
-        <v>231</v>
+        <v>336</v>
       </c>
       <c r="C85" t="s">
-        <v>227</v>
+        <v>171</v>
       </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B86" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C86" t="s">
         <v>171</v>
@@ -2546,10 +2585,10 @@
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B87" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C87" t="s">
         <v>171</v>
@@ -2557,10 +2596,10 @@
     </row>
     <row r="88" spans="1:3">
       <c r="A88" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B88" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="C88" t="s">
         <v>171</v>
@@ -2582,29 +2621,29 @@
         <v>344</v>
       </c>
       <c r="B90" t="s">
-        <v>345</v>
+        <v>234</v>
       </c>
       <c r="C90" t="s">
-        <v>171</v>
+        <v>230</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
+        <v>345</v>
+      </c>
+      <c r="B91" t="s">
         <v>346</v>
       </c>
-      <c r="B91" t="s">
-        <v>347</v>
-      </c>
       <c r="C91" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" t="s">
+        <v>347</v>
+      </c>
+      <c r="B92" t="s">
         <v>348</v>
-      </c>
-      <c r="B92" t="s">
-        <v>349</v>
       </c>
       <c r="C92" t="s">
         <v>171</v>
@@ -2612,10 +2651,10 @@
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
+        <v>349</v>
+      </c>
+      <c r="B93" t="s">
         <v>350</v>
-      </c>
-      <c r="B93" t="s">
-        <v>351</v>
       </c>
       <c r="C93" t="s">
         <v>171</v>
@@ -2623,10 +2662,10 @@
     </row>
     <row r="94" spans="1:3">
       <c r="A94" t="s">
+        <v>351</v>
+      </c>
+      <c r="B94" t="s">
         <v>352</v>
-      </c>
-      <c r="B94" t="s">
-        <v>353</v>
       </c>
       <c r="C94" t="s">
         <v>171</v>
@@ -2634,10 +2673,10 @@
     </row>
     <row r="95" spans="1:3">
       <c r="A95" t="s">
+        <v>353</v>
+      </c>
+      <c r="B95" t="s">
         <v>354</v>
-      </c>
-      <c r="B95" t="s">
-        <v>355</v>
       </c>
       <c r="C95" t="s">
         <v>171</v>
@@ -2645,13 +2684,13 @@
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
+        <v>355</v>
+      </c>
+      <c r="B96" t="s">
         <v>356</v>
       </c>
-      <c r="B96" t="s">
-        <v>170</v>
-      </c>
       <c r="C96" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
     </row>
     <row r="97" spans="1:3">
@@ -2703,7 +2742,7 @@
         <v>365</v>
       </c>
       <c r="B101" t="s">
-        <v>366</v>
+        <v>170</v>
       </c>
       <c r="C101" t="s">
         <v>171</v>
@@ -2711,10 +2750,10 @@
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
+        <v>366</v>
+      </c>
+      <c r="B102" t="s">
         <v>367</v>
-      </c>
-      <c r="B102" t="s">
-        <v>216</v>
       </c>
       <c r="C102" t="s">
         <v>171</v>
@@ -2769,7 +2808,7 @@
         <v>376</v>
       </c>
       <c r="B107" t="s">
-        <v>377</v>
+        <v>216</v>
       </c>
       <c r="C107" t="s">
         <v>171</v>
@@ -2777,12 +2816,89 @@
     </row>
     <row r="108" spans="1:3">
       <c r="A108" t="s">
+        <v>377</v>
+      </c>
+      <c r="B108" t="s">
         <v>378</v>
       </c>
-      <c r="B108" t="s">
+      <c r="C108" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3">
+      <c r="A109" t="s">
         <v>379</v>
       </c>
-      <c r="C108" t="s">
+      <c r="B109" t="s">
+        <v>380</v>
+      </c>
+      <c r="C109" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3">
+      <c r="A110" t="s">
+        <v>381</v>
+      </c>
+      <c r="B110" t="s">
+        <v>382</v>
+      </c>
+      <c r="C110" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3">
+      <c r="A111" t="s">
+        <v>383</v>
+      </c>
+      <c r="B111" t="s">
+        <v>384</v>
+      </c>
+      <c r="C111" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3">
+      <c r="A112" t="s">
+        <v>385</v>
+      </c>
+      <c r="B112" t="s">
+        <v>386</v>
+      </c>
+      <c r="C112" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3">
+      <c r="A113" t="s">
+        <v>387</v>
+      </c>
+      <c r="B113" t="s">
+        <v>388</v>
+      </c>
+      <c r="C113" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3">
+      <c r="A114" t="s">
+        <v>389</v>
+      </c>
+      <c r="B114" t="s">
+        <v>390</v>
+      </c>
+      <c r="C114" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3">
+      <c r="A115" t="s">
+        <v>391</v>
+      </c>
+      <c r="B115" t="s">
+        <v>392</v>
+      </c>
+      <c r="C115" t="s">
         <v>171</v>
       </c>
     </row>

</xml_diff>